<commit_message>
Fix workbook crossing checks
Co-authored-by: bvn2103 <318941354+bvn2103@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/capabilities/marginal-analysis/model.xlsx
+++ b/capabilities/marginal-analysis/model.xlsx
@@ -995,7 +995,7 @@
         <v/>
       </c>
       <c r="C5" s="11">
-        <f>MIN(H12:H32)</f>
+        <f>IF(COUNT(H12:H32)=0,"",MINIFS(H12:H32,H12:H32,"&gt;0"))</f>
         <v/>
       </c>
       <c r="D5" s="11">
@@ -1014,7 +1014,7 @@
         <v/>
       </c>
       <c r="C6" s="11">
-        <f>MIN(H34:H64)</f>
+        <f>IF(COUNT(H34:H64)=0,"",MINIFS(H34:H64,H34:H64,"&gt;0"))</f>
         <v/>
       </c>
       <c r="D6" s="11">
@@ -1033,7 +1033,7 @@
         <v/>
       </c>
       <c r="C7" s="11">
-        <f>MIN(H66:H86)</f>
+        <f>IF(COUNT(H66:H86)=0,"",MINIFS(H66:H86,H66:H86,"&gt;0"))</f>
         <v/>
       </c>
       <c r="D7" s="11">
@@ -1147,7 +1147,7 @@
         <v/>
       </c>
       <c r="H13" s="14">
-        <f>IF(AND(F13&gt;G13,F12&lt;=G12),B13,"")</f>
+        <f>IF(AND(F13&gt;G13,F12&lt;=G13),B13,"")</f>
         <v/>
       </c>
     </row>
@@ -1181,7 +1181,7 @@
         <v/>
       </c>
       <c r="H14" s="14">
-        <f>IF(AND(F14&gt;G14,F13&lt;=G13),B14,"")</f>
+        <f>IF(AND(F14&gt;G14,F13&lt;=G14),B14,"")</f>
         <v/>
       </c>
     </row>
@@ -1215,7 +1215,7 @@
         <v/>
       </c>
       <c r="H15" s="14">
-        <f>IF(AND(F15&gt;G15,F14&lt;=G14),B15,"")</f>
+        <f>IF(AND(F15&gt;G15,F14&lt;=G15),B15,"")</f>
         <v/>
       </c>
     </row>
@@ -1249,7 +1249,7 @@
         <v/>
       </c>
       <c r="H16" s="14">
-        <f>IF(AND(F16&gt;G16,F15&lt;=G15),B16,"")</f>
+        <f>IF(AND(F16&gt;G16,F15&lt;=G16),B16,"")</f>
         <v/>
       </c>
     </row>
@@ -1283,7 +1283,7 @@
         <v/>
       </c>
       <c r="H17" s="14">
-        <f>IF(AND(F17&gt;G17,F16&lt;=G16),B17,"")</f>
+        <f>IF(AND(F17&gt;G17,F16&lt;=G17),B17,"")</f>
         <v/>
       </c>
     </row>
@@ -1317,7 +1317,7 @@
         <v/>
       </c>
       <c r="H18" s="14">
-        <f>IF(AND(F18&gt;G18,F17&lt;=G17),B18,"")</f>
+        <f>IF(AND(F18&gt;G18,F17&lt;=G18),B18,"")</f>
         <v/>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
         <v/>
       </c>
       <c r="H19" s="14">
-        <f>IF(AND(F19&gt;G19,F18&lt;=G18),B19,"")</f>
+        <f>IF(AND(F19&gt;G19,F18&lt;=G19),B19,"")</f>
         <v/>
       </c>
     </row>
@@ -1385,7 +1385,7 @@
         <v/>
       </c>
       <c r="H20" s="14">
-        <f>IF(AND(F20&gt;G20,F19&lt;=G19),B20,"")</f>
+        <f>IF(AND(F20&gt;G20,F19&lt;=G20),B20,"")</f>
         <v/>
       </c>
     </row>
@@ -1419,7 +1419,7 @@
         <v/>
       </c>
       <c r="H21" s="14">
-        <f>IF(AND(F21&gt;G21,F20&lt;=G20),B21,"")</f>
+        <f>IF(AND(F21&gt;G21,F20&lt;=G21),B21,"")</f>
         <v/>
       </c>
     </row>
@@ -1453,7 +1453,7 @@
         <v/>
       </c>
       <c r="H22" s="14">
-        <f>IF(AND(F22&gt;G22,F21&lt;=G21),B22,"")</f>
+        <f>IF(AND(F22&gt;G22,F21&lt;=G22),B22,"")</f>
         <v/>
       </c>
     </row>
@@ -1487,7 +1487,7 @@
         <v/>
       </c>
       <c r="H23" s="14">
-        <f>IF(AND(F23&gt;G23,F22&lt;=G22),B23,"")</f>
+        <f>IF(AND(F23&gt;G23,F22&lt;=G23),B23,"")</f>
         <v/>
       </c>
     </row>
@@ -1521,7 +1521,7 @@
         <v/>
       </c>
       <c r="H24" s="14">
-        <f>IF(AND(F24&gt;G24,F23&lt;=G23),B24,"")</f>
+        <f>IF(AND(F24&gt;G24,F23&lt;=G24),B24,"")</f>
         <v/>
       </c>
     </row>
@@ -1555,7 +1555,7 @@
         <v/>
       </c>
       <c r="H25" s="14">
-        <f>IF(AND(F25&gt;G25,F24&lt;=G24),B25,"")</f>
+        <f>IF(AND(F25&gt;G25,F24&lt;=G25),B25,"")</f>
         <v/>
       </c>
     </row>
@@ -1589,7 +1589,7 @@
         <v/>
       </c>
       <c r="H26" s="14">
-        <f>IF(AND(F26&gt;G26,F25&lt;=G25),B26,"")</f>
+        <f>IF(AND(F26&gt;G26,F25&lt;=G26),B26,"")</f>
         <v/>
       </c>
     </row>
@@ -1623,7 +1623,7 @@
         <v/>
       </c>
       <c r="H27" s="14">
-        <f>IF(AND(F27&gt;G27,F26&lt;=G26),B27,"")</f>
+        <f>IF(AND(F27&gt;G27,F26&lt;=G27),B27,"")</f>
         <v/>
       </c>
     </row>
@@ -1657,7 +1657,7 @@
         <v/>
       </c>
       <c r="H28" s="14">
-        <f>IF(AND(F28&gt;G28,F27&lt;=G27),B28,"")</f>
+        <f>IF(AND(F28&gt;G28,F27&lt;=G28),B28,"")</f>
         <v/>
       </c>
     </row>
@@ -1691,7 +1691,7 @@
         <v/>
       </c>
       <c r="H29" s="14">
-        <f>IF(AND(F29&gt;G29,F28&lt;=G28),B29,"")</f>
+        <f>IF(AND(F29&gt;G29,F28&lt;=G29),B29,"")</f>
         <v/>
       </c>
     </row>
@@ -1725,7 +1725,7 @@
         <v/>
       </c>
       <c r="H30" s="14">
-        <f>IF(AND(F30&gt;G30,F29&lt;=G29),B30,"")</f>
+        <f>IF(AND(F30&gt;G30,F29&lt;=G30),B30,"")</f>
         <v/>
       </c>
     </row>
@@ -1759,7 +1759,7 @@
         <v/>
       </c>
       <c r="H31" s="14">
-        <f>IF(AND(F31&gt;G31,F30&lt;=G30),B31,"")</f>
+        <f>IF(AND(F31&gt;G31,F30&lt;=G31),B31,"")</f>
         <v/>
       </c>
     </row>
@@ -1793,7 +1793,7 @@
         <v/>
       </c>
       <c r="H32" s="14">
-        <f>IF(AND(F32&gt;G32,F31&lt;=G31),B32,"")</f>
+        <f>IF(AND(F32&gt;G32,F31&lt;=G32),B32,"")</f>
         <v/>
       </c>
     </row>
@@ -1861,7 +1861,7 @@
         <v/>
       </c>
       <c r="H35" s="14">
-        <f>IF(AND(F35&gt;G35,F34&lt;=G34),B35,"")</f>
+        <f>IF(AND(F35&gt;G35,F34&lt;=G35),B35,"")</f>
         <v/>
       </c>
     </row>
@@ -1895,7 +1895,7 @@
         <v/>
       </c>
       <c r="H36" s="14">
-        <f>IF(AND(F36&gt;G36,F35&lt;=G35),B36,"")</f>
+        <f>IF(AND(F36&gt;G36,F35&lt;=G36),B36,"")</f>
         <v/>
       </c>
     </row>
@@ -1929,7 +1929,7 @@
         <v/>
       </c>
       <c r="H37" s="14">
-        <f>IF(AND(F37&gt;G37,F36&lt;=G36),B37,"")</f>
+        <f>IF(AND(F37&gt;G37,F36&lt;=G37),B37,"")</f>
         <v/>
       </c>
     </row>
@@ -1963,7 +1963,7 @@
         <v/>
       </c>
       <c r="H38" s="14">
-        <f>IF(AND(F38&gt;G38,F37&lt;=G37),B38,"")</f>
+        <f>IF(AND(F38&gt;G38,F37&lt;=G38),B38,"")</f>
         <v/>
       </c>
     </row>
@@ -1997,7 +1997,7 @@
         <v/>
       </c>
       <c r="H39" s="14">
-        <f>IF(AND(F39&gt;G39,F38&lt;=G38),B39,"")</f>
+        <f>IF(AND(F39&gt;G39,F38&lt;=G39),B39,"")</f>
         <v/>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
         <v/>
       </c>
       <c r="H40" s="14">
-        <f>IF(AND(F40&gt;G40,F39&lt;=G39),B40,"")</f>
+        <f>IF(AND(F40&gt;G40,F39&lt;=G40),B40,"")</f>
         <v/>
       </c>
     </row>
@@ -2065,7 +2065,7 @@
         <v/>
       </c>
       <c r="H41" s="14">
-        <f>IF(AND(F41&gt;G41,F40&lt;=G40),B41,"")</f>
+        <f>IF(AND(F41&gt;G41,F40&lt;=G41),B41,"")</f>
         <v/>
       </c>
     </row>
@@ -2099,7 +2099,7 @@
         <v/>
       </c>
       <c r="H42" s="14">
-        <f>IF(AND(F42&gt;G42,F41&lt;=G41),B42,"")</f>
+        <f>IF(AND(F42&gt;G42,F41&lt;=G42),B42,"")</f>
         <v/>
       </c>
     </row>
@@ -2133,7 +2133,7 @@
         <v/>
       </c>
       <c r="H43" s="14">
-        <f>IF(AND(F43&gt;G43,F42&lt;=G42),B43,"")</f>
+        <f>IF(AND(F43&gt;G43,F42&lt;=G43),B43,"")</f>
         <v/>
       </c>
     </row>
@@ -2167,7 +2167,7 @@
         <v/>
       </c>
       <c r="H44" s="14">
-        <f>IF(AND(F44&gt;G44,F43&lt;=G43),B44,"")</f>
+        <f>IF(AND(F44&gt;G44,F43&lt;=G44),B44,"")</f>
         <v/>
       </c>
     </row>
@@ -2201,7 +2201,7 @@
         <v/>
       </c>
       <c r="H45" s="14">
-        <f>IF(AND(F45&gt;G45,F44&lt;=G44),B45,"")</f>
+        <f>IF(AND(F45&gt;G45,F44&lt;=G45),B45,"")</f>
         <v/>
       </c>
     </row>
@@ -2235,7 +2235,7 @@
         <v/>
       </c>
       <c r="H46" s="14">
-        <f>IF(AND(F46&gt;G46,F45&lt;=G45),B46,"")</f>
+        <f>IF(AND(F46&gt;G46,F45&lt;=G46),B46,"")</f>
         <v/>
       </c>
     </row>
@@ -2269,7 +2269,7 @@
         <v/>
       </c>
       <c r="H47" s="14">
-        <f>IF(AND(F47&gt;G47,F46&lt;=G46),B47,"")</f>
+        <f>IF(AND(F47&gt;G47,F46&lt;=G47),B47,"")</f>
         <v/>
       </c>
     </row>
@@ -2303,7 +2303,7 @@
         <v/>
       </c>
       <c r="H48" s="14">
-        <f>IF(AND(F48&gt;G48,F47&lt;=G47),B48,"")</f>
+        <f>IF(AND(F48&gt;G48,F47&lt;=G48),B48,"")</f>
         <v/>
       </c>
     </row>
@@ -2337,7 +2337,7 @@
         <v/>
       </c>
       <c r="H49" s="14">
-        <f>IF(AND(F49&gt;G49,F48&lt;=G48),B49,"")</f>
+        <f>IF(AND(F49&gt;G49,F48&lt;=G49),B49,"")</f>
         <v/>
       </c>
     </row>
@@ -2371,7 +2371,7 @@
         <v/>
       </c>
       <c r="H50" s="14">
-        <f>IF(AND(F50&gt;G50,F49&lt;=G49),B50,"")</f>
+        <f>IF(AND(F50&gt;G50,F49&lt;=G50),B50,"")</f>
         <v/>
       </c>
     </row>
@@ -2405,7 +2405,7 @@
         <v/>
       </c>
       <c r="H51" s="14">
-        <f>IF(AND(F51&gt;G51,F50&lt;=G50),B51,"")</f>
+        <f>IF(AND(F51&gt;G51,F50&lt;=G51),B51,"")</f>
         <v/>
       </c>
     </row>
@@ -2439,7 +2439,7 @@
         <v/>
       </c>
       <c r="H52" s="14">
-        <f>IF(AND(F52&gt;G52,F51&lt;=G51),B52,"")</f>
+        <f>IF(AND(F52&gt;G52,F51&lt;=G52),B52,"")</f>
         <v/>
       </c>
     </row>
@@ -2473,7 +2473,7 @@
         <v/>
       </c>
       <c r="H53" s="14">
-        <f>IF(AND(F53&gt;G53,F52&lt;=G52),B53,"")</f>
+        <f>IF(AND(F53&gt;G53,F52&lt;=G53),B53,"")</f>
         <v/>
       </c>
     </row>
@@ -2507,7 +2507,7 @@
         <v/>
       </c>
       <c r="H54" s="14">
-        <f>IF(AND(F54&gt;G54,F53&lt;=G53),B54,"")</f>
+        <f>IF(AND(F54&gt;G54,F53&lt;=G54),B54,"")</f>
         <v/>
       </c>
     </row>
@@ -2541,7 +2541,7 @@
         <v/>
       </c>
       <c r="H55" s="14">
-        <f>IF(AND(F55&gt;G55,F54&lt;=G54),B55,"")</f>
+        <f>IF(AND(F55&gt;G55,F54&lt;=G55),B55,"")</f>
         <v/>
       </c>
     </row>
@@ -2575,7 +2575,7 @@
         <v/>
       </c>
       <c r="H56" s="14">
-        <f>IF(AND(F56&gt;G56,F55&lt;=G55),B56,"")</f>
+        <f>IF(AND(F56&gt;G56,F55&lt;=G56),B56,"")</f>
         <v/>
       </c>
     </row>
@@ -2609,7 +2609,7 @@
         <v/>
       </c>
       <c r="H57" s="14">
-        <f>IF(AND(F57&gt;G57,F56&lt;=G56),B57,"")</f>
+        <f>IF(AND(F57&gt;G57,F56&lt;=G57),B57,"")</f>
         <v/>
       </c>
     </row>
@@ -2643,7 +2643,7 @@
         <v/>
       </c>
       <c r="H58" s="14">
-        <f>IF(AND(F58&gt;G58,F57&lt;=G57),B58,"")</f>
+        <f>IF(AND(F58&gt;G58,F57&lt;=G58),B58,"")</f>
         <v/>
       </c>
     </row>
@@ -2677,7 +2677,7 @@
         <v/>
       </c>
       <c r="H59" s="14">
-        <f>IF(AND(F59&gt;G59,F58&lt;=G58),B59,"")</f>
+        <f>IF(AND(F59&gt;G59,F58&lt;=G59),B59,"")</f>
         <v/>
       </c>
     </row>
@@ -2711,7 +2711,7 @@
         <v/>
       </c>
       <c r="H60" s="14">
-        <f>IF(AND(F60&gt;G60,F59&lt;=G59),B60,"")</f>
+        <f>IF(AND(F60&gt;G60,F59&lt;=G60),B60,"")</f>
         <v/>
       </c>
     </row>
@@ -2745,7 +2745,7 @@
         <v/>
       </c>
       <c r="H61" s="14">
-        <f>IF(AND(F61&gt;G61,F60&lt;=G60),B61,"")</f>
+        <f>IF(AND(F61&gt;G61,F60&lt;=G61),B61,"")</f>
         <v/>
       </c>
     </row>
@@ -2779,7 +2779,7 @@
         <v/>
       </c>
       <c r="H62" s="14">
-        <f>IF(AND(F62&gt;G62,F61&lt;=G61),B62,"")</f>
+        <f>IF(AND(F62&gt;G62,F61&lt;=G62),B62,"")</f>
         <v/>
       </c>
     </row>
@@ -2813,7 +2813,7 @@
         <v/>
       </c>
       <c r="H63" s="14">
-        <f>IF(AND(F63&gt;G63,F62&lt;=G62),B63,"")</f>
+        <f>IF(AND(F63&gt;G63,F62&lt;=G63),B63,"")</f>
         <v/>
       </c>
     </row>
@@ -2847,7 +2847,7 @@
         <v/>
       </c>
       <c r="H64" s="14">
-        <f>IF(AND(F64&gt;G64,F63&lt;=G63),B64,"")</f>
+        <f>IF(AND(F64&gt;G64,F63&lt;=G64),B64,"")</f>
         <v/>
       </c>
     </row>
@@ -2915,7 +2915,7 @@
         <v/>
       </c>
       <c r="H67" s="14">
-        <f>IF(AND(F67&gt;G67,F66&lt;=G66),B67,"")</f>
+        <f>IF(AND(F67&gt;G67,F66&lt;=G67),B67,"")</f>
         <v/>
       </c>
     </row>
@@ -2949,7 +2949,7 @@
         <v/>
       </c>
       <c r="H68" s="14">
-        <f>IF(AND(F68&gt;G68,F67&lt;=G67),B68,"")</f>
+        <f>IF(AND(F68&gt;G68,F67&lt;=G68),B68,"")</f>
         <v/>
       </c>
     </row>
@@ -2983,7 +2983,7 @@
         <v/>
       </c>
       <c r="H69" s="14">
-        <f>IF(AND(F69&gt;G69,F68&lt;=G68),B69,"")</f>
+        <f>IF(AND(F69&gt;G69,F68&lt;=G69),B69,"")</f>
         <v/>
       </c>
     </row>
@@ -3017,7 +3017,7 @@
         <v/>
       </c>
       <c r="H70" s="14">
-        <f>IF(AND(F70&gt;G70,F69&lt;=G69),B70,"")</f>
+        <f>IF(AND(F70&gt;G70,F69&lt;=G70),B70,"")</f>
         <v/>
       </c>
     </row>
@@ -3051,7 +3051,7 @@
         <v/>
       </c>
       <c r="H71" s="14">
-        <f>IF(AND(F71&gt;G71,F70&lt;=G70),B71,"")</f>
+        <f>IF(AND(F71&gt;G71,F70&lt;=G71),B71,"")</f>
         <v/>
       </c>
     </row>
@@ -3085,7 +3085,7 @@
         <v/>
       </c>
       <c r="H72" s="14">
-        <f>IF(AND(F72&gt;G72,F71&lt;=G71),B72,"")</f>
+        <f>IF(AND(F72&gt;G72,F71&lt;=G72),B72,"")</f>
         <v/>
       </c>
     </row>
@@ -3119,7 +3119,7 @@
         <v/>
       </c>
       <c r="H73" s="14">
-        <f>IF(AND(F73&gt;G73,F72&lt;=G72),B73,"")</f>
+        <f>IF(AND(F73&gt;G73,F72&lt;=G73),B73,"")</f>
         <v/>
       </c>
     </row>
@@ -3153,7 +3153,7 @@
         <v/>
       </c>
       <c r="H74" s="14">
-        <f>IF(AND(F74&gt;G74,F73&lt;=G73),B74,"")</f>
+        <f>IF(AND(F74&gt;G74,F73&lt;=G74),B74,"")</f>
         <v/>
       </c>
     </row>
@@ -3187,7 +3187,7 @@
         <v/>
       </c>
       <c r="H75" s="14">
-        <f>IF(AND(F75&gt;G75,F74&lt;=G74),B75,"")</f>
+        <f>IF(AND(F75&gt;G75,F74&lt;=G75),B75,"")</f>
         <v/>
       </c>
     </row>
@@ -3221,7 +3221,7 @@
         <v/>
       </c>
       <c r="H76" s="14">
-        <f>IF(AND(F76&gt;G76,F75&lt;=G75),B76,"")</f>
+        <f>IF(AND(F76&gt;G76,F75&lt;=G76),B76,"")</f>
         <v/>
       </c>
     </row>
@@ -3255,7 +3255,7 @@
         <v/>
       </c>
       <c r="H77" s="14">
-        <f>IF(AND(F77&gt;G77,F76&lt;=G76),B77,"")</f>
+        <f>IF(AND(F77&gt;G77,F76&lt;=G77),B77,"")</f>
         <v/>
       </c>
     </row>
@@ -3289,7 +3289,7 @@
         <v/>
       </c>
       <c r="H78" s="14">
-        <f>IF(AND(F78&gt;G78,F77&lt;=G77),B78,"")</f>
+        <f>IF(AND(F78&gt;G78,F77&lt;=G78),B78,"")</f>
         <v/>
       </c>
     </row>
@@ -3323,7 +3323,7 @@
         <v/>
       </c>
       <c r="H79" s="14">
-        <f>IF(AND(F79&gt;G79,F78&lt;=G78),B79,"")</f>
+        <f>IF(AND(F79&gt;G79,F78&lt;=G79),B79,"")</f>
         <v/>
       </c>
     </row>
@@ -3357,7 +3357,7 @@
         <v/>
       </c>
       <c r="H80" s="14">
-        <f>IF(AND(F80&gt;G80,F79&lt;=G79),B80,"")</f>
+        <f>IF(AND(F80&gt;G80,F79&lt;=G80),B80,"")</f>
         <v/>
       </c>
     </row>
@@ -3391,7 +3391,7 @@
         <v/>
       </c>
       <c r="H81" s="14">
-        <f>IF(AND(F81&gt;G81,F80&lt;=G80),B81,"")</f>
+        <f>IF(AND(F81&gt;G81,F80&lt;=G81),B81,"")</f>
         <v/>
       </c>
     </row>
@@ -3425,7 +3425,7 @@
         <v/>
       </c>
       <c r="H82" s="14">
-        <f>IF(AND(F82&gt;G82,F81&lt;=G81),B82,"")</f>
+        <f>IF(AND(F82&gt;G82,F81&lt;=G82),B82,"")</f>
         <v/>
       </c>
     </row>
@@ -3459,7 +3459,7 @@
         <v/>
       </c>
       <c r="H83" s="14">
-        <f>IF(AND(F83&gt;G83,F82&lt;=G82),B83,"")</f>
+        <f>IF(AND(F83&gt;G83,F82&lt;=G83),B83,"")</f>
         <v/>
       </c>
     </row>
@@ -3493,7 +3493,7 @@
         <v/>
       </c>
       <c r="H84" s="14">
-        <f>IF(AND(F84&gt;G84,F83&lt;=G83),B84,"")</f>
+        <f>IF(AND(F84&gt;G84,F83&lt;=G84),B84,"")</f>
         <v/>
       </c>
     </row>
@@ -3527,7 +3527,7 @@
         <v/>
       </c>
       <c r="H85" s="14">
-        <f>IF(AND(F85&gt;G85,F84&lt;=G84),B85,"")</f>
+        <f>IF(AND(F85&gt;G85,F84&lt;=G85),B85,"")</f>
         <v/>
       </c>
     </row>
@@ -3561,7 +3561,7 @@
         <v/>
       </c>
       <c r="H86" s="14">
-        <f>IF(AND(F86&gt;G86,F85&lt;=G85),B86,"")</f>
+        <f>IF(AND(F86&gt;G86,F85&lt;=G86),B86,"")</f>
         <v/>
       </c>
     </row>
@@ -4214,10 +4214,10 @@
   </sheetData>
   <conditionalFormatting sqref="D5:D18">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>$D5="PASS"</formula>
+      <formula>EXACT($D5,"PASS")</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="1">
-      <formula>$D5="FAIL"</formula>
+      <formula>EXACT($D5,"FAIL")</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Improve workbook Excel compatibility
Co-authored-by: bvn2103 <318941354+bvn2103@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/capabilities/marginal-analysis/model.xlsx
+++ b/capabilities/marginal-analysis/model.xlsx
@@ -995,7 +995,7 @@
         <v/>
       </c>
       <c r="C5" s="11">
-        <f>IF(COUNT(H12:H32)=0,"",MINIFS(H12:H32,H12:H32,"&gt;0"))</f>
+        <f>IF(COUNT(H12:H32)=0,"",AGGREGATE(15,6,H12:H32/(H12:H32&gt;0),1))</f>
         <v/>
       </c>
       <c r="D5" s="11">
@@ -1014,7 +1014,7 @@
         <v/>
       </c>
       <c r="C6" s="11">
-        <f>IF(COUNT(H34:H64)=0,"",MINIFS(H34:H64,H34:H64,"&gt;0"))</f>
+        <f>IF(COUNT(H34:H64)=0,"",AGGREGATE(15,6,H34:H64/(H34:H64&gt;0),1))</f>
         <v/>
       </c>
       <c r="D6" s="11">
@@ -1033,7 +1033,7 @@
         <v/>
       </c>
       <c r="C7" s="11">
-        <f>IF(COUNT(H66:H86)=0,"",MINIFS(H66:H86,H66:H86,"&gt;0"))</f>
+        <f>IF(COUNT(H66:H86)=0,"",AGGREGATE(15,6,H66:H86/(H66:H86&gt;0),1))</f>
         <v/>
       </c>
       <c r="D7" s="11">

</xml_diff>

<commit_message>
Refine workbook summary formatting
Co-authored-by: bvn2103 <318941354+bvn2103@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/capabilities/marginal-analysis/model.xlsx
+++ b/capabilities/marginal-analysis/model.xlsx
@@ -64,7 +64,7 @@
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.000000"/>
     <numFmt numFmtId="166" formatCode="0.0000%"/>
-    <numFmt numFmtId="167" formatCode="$#,##0.0000"/>
+    <numFmt numFmtId="167" formatCode="0.0000"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -3863,7 +3863,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Blended labor rate</t>
+          <t>Blended labor rate ($/hour)</t>
         </is>
       </c>
       <c r="B16" s="18">
@@ -4230,7 +4230,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4413,21 +4413,32 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Fixed cost</t>
-        </is>
-      </c>
-      <c r="B14" s="10">
-        <f>Fixed_Cost</f>
+          <t>Blended labor rate ($/hour)</t>
+        </is>
+      </c>
+      <c r="B14" s="18">
+        <f>Blended_Labor_Rate</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
+          <t>Fixed cost</t>
+        </is>
+      </c>
+      <c r="B15" s="10">
+        <f>Fixed_Cost</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
           <t>Profit</t>
         </is>
       </c>
-      <c r="B15" s="10">
+      <c r="B16" s="10">
         <f>Profit</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Tighten workbook crossing logic
Co-authored-by: bvn2103 <318941354+bvn2103@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/capabilities/marginal-analysis/model.xlsx
+++ b/capabilities/marginal-analysis/model.xlsx
@@ -995,7 +995,7 @@
         <v/>
       </c>
       <c r="C5" s="11">
-        <f>IF(COUNT(H12:H32)=0,"",AGGREGATE(15,6,H12:H32/(H12:H32&gt;0),1))</f>
+        <f>IF(COUNT(H12:H32)=0,"",SUM(H12:H32))</f>
         <v/>
       </c>
       <c r="D5" s="11">
@@ -1014,7 +1014,7 @@
         <v/>
       </c>
       <c r="C6" s="11">
-        <f>IF(COUNT(H34:H64)=0,"",AGGREGATE(15,6,H34:H64/(H34:H64&gt;0),1))</f>
+        <f>IF(COUNT(H34:H64)=0,"",SUM(H34:H64))</f>
         <v/>
       </c>
       <c r="D6" s="11">
@@ -1033,7 +1033,7 @@
         <v/>
       </c>
       <c r="C7" s="11">
-        <f>IF(COUNT(H66:H86)=0,"",AGGREGATE(15,6,H66:H86/(H66:H86&gt;0),1))</f>
+        <f>IF(COUNT(H66:H86)=0,"",SUM(H66:H86))</f>
         <v/>
       </c>
       <c r="D7" s="11">
@@ -1147,7 +1147,7 @@
         <v/>
       </c>
       <c r="H13" s="14">
-        <f>IF(AND(F13&gt;G13,F12&lt;=G13),B13,"")</f>
+        <f>IF(AND(F13&gt;G13,COUNT(H12:H12)=0),B13,"")</f>
         <v/>
       </c>
     </row>
@@ -1181,7 +1181,7 @@
         <v/>
       </c>
       <c r="H14" s="14">
-        <f>IF(AND(F14&gt;G14,F13&lt;=G14),B14,"")</f>
+        <f>IF(AND(F14&gt;G14,COUNT(H12:H13)=0),B14,"")</f>
         <v/>
       </c>
     </row>
@@ -1215,7 +1215,7 @@
         <v/>
       </c>
       <c r="H15" s="14">
-        <f>IF(AND(F15&gt;G15,F14&lt;=G15),B15,"")</f>
+        <f>IF(AND(F15&gt;G15,COUNT(H12:H14)=0),B15,"")</f>
         <v/>
       </c>
     </row>
@@ -1249,7 +1249,7 @@
         <v/>
       </c>
       <c r="H16" s="14">
-        <f>IF(AND(F16&gt;G16,F15&lt;=G16),B16,"")</f>
+        <f>IF(AND(F16&gt;G16,COUNT(H12:H15)=0),B16,"")</f>
         <v/>
       </c>
     </row>
@@ -1283,7 +1283,7 @@
         <v/>
       </c>
       <c r="H17" s="14">
-        <f>IF(AND(F17&gt;G17,F16&lt;=G17),B17,"")</f>
+        <f>IF(AND(F17&gt;G17,COUNT(H12:H16)=0),B17,"")</f>
         <v/>
       </c>
     </row>
@@ -1317,7 +1317,7 @@
         <v/>
       </c>
       <c r="H18" s="14">
-        <f>IF(AND(F18&gt;G18,F17&lt;=G18),B18,"")</f>
+        <f>IF(AND(F18&gt;G18,COUNT(H12:H17)=0),B18,"")</f>
         <v/>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
         <v/>
       </c>
       <c r="H19" s="14">
-        <f>IF(AND(F19&gt;G19,F18&lt;=G19),B19,"")</f>
+        <f>IF(AND(F19&gt;G19,COUNT(H12:H18)=0),B19,"")</f>
         <v/>
       </c>
     </row>
@@ -1385,7 +1385,7 @@
         <v/>
       </c>
       <c r="H20" s="14">
-        <f>IF(AND(F20&gt;G20,F19&lt;=G20),B20,"")</f>
+        <f>IF(AND(F20&gt;G20,COUNT(H12:H19)=0),B20,"")</f>
         <v/>
       </c>
     </row>
@@ -1419,7 +1419,7 @@
         <v/>
       </c>
       <c r="H21" s="14">
-        <f>IF(AND(F21&gt;G21,F20&lt;=G21),B21,"")</f>
+        <f>IF(AND(F21&gt;G21,COUNT(H12:H20)=0),B21,"")</f>
         <v/>
       </c>
     </row>
@@ -1453,7 +1453,7 @@
         <v/>
       </c>
       <c r="H22" s="14">
-        <f>IF(AND(F22&gt;G22,F21&lt;=G22),B22,"")</f>
+        <f>IF(AND(F22&gt;G22,COUNT(H12:H21)=0),B22,"")</f>
         <v/>
       </c>
     </row>
@@ -1487,7 +1487,7 @@
         <v/>
       </c>
       <c r="H23" s="14">
-        <f>IF(AND(F23&gt;G23,F22&lt;=G23),B23,"")</f>
+        <f>IF(AND(F23&gt;G23,COUNT(H12:H22)=0),B23,"")</f>
         <v/>
       </c>
     </row>
@@ -1521,7 +1521,7 @@
         <v/>
       </c>
       <c r="H24" s="14">
-        <f>IF(AND(F24&gt;G24,F23&lt;=G24),B24,"")</f>
+        <f>IF(AND(F24&gt;G24,COUNT(H12:H23)=0),B24,"")</f>
         <v/>
       </c>
     </row>
@@ -1555,7 +1555,7 @@
         <v/>
       </c>
       <c r="H25" s="14">
-        <f>IF(AND(F25&gt;G25,F24&lt;=G25),B25,"")</f>
+        <f>IF(AND(F25&gt;G25,COUNT(H12:H24)=0),B25,"")</f>
         <v/>
       </c>
     </row>
@@ -1589,7 +1589,7 @@
         <v/>
       </c>
       <c r="H26" s="14">
-        <f>IF(AND(F26&gt;G26,F25&lt;=G26),B26,"")</f>
+        <f>IF(AND(F26&gt;G26,COUNT(H12:H25)=0),B26,"")</f>
         <v/>
       </c>
     </row>
@@ -1623,7 +1623,7 @@
         <v/>
       </c>
       <c r="H27" s="14">
-        <f>IF(AND(F27&gt;G27,F26&lt;=G27),B27,"")</f>
+        <f>IF(AND(F27&gt;G27,COUNT(H12:H26)=0),B27,"")</f>
         <v/>
       </c>
     </row>
@@ -1657,7 +1657,7 @@
         <v/>
       </c>
       <c r="H28" s="14">
-        <f>IF(AND(F28&gt;G28,F27&lt;=G28),B28,"")</f>
+        <f>IF(AND(F28&gt;G28,COUNT(H12:H27)=0),B28,"")</f>
         <v/>
       </c>
     </row>
@@ -1691,7 +1691,7 @@
         <v/>
       </c>
       <c r="H29" s="14">
-        <f>IF(AND(F29&gt;G29,F28&lt;=G29),B29,"")</f>
+        <f>IF(AND(F29&gt;G29,COUNT(H12:H28)=0),B29,"")</f>
         <v/>
       </c>
     </row>
@@ -1725,7 +1725,7 @@
         <v/>
       </c>
       <c r="H30" s="14">
-        <f>IF(AND(F30&gt;G30,F29&lt;=G30),B30,"")</f>
+        <f>IF(AND(F30&gt;G30,COUNT(H12:H29)=0),B30,"")</f>
         <v/>
       </c>
     </row>
@@ -1759,7 +1759,7 @@
         <v/>
       </c>
       <c r="H31" s="14">
-        <f>IF(AND(F31&gt;G31,F30&lt;=G31),B31,"")</f>
+        <f>IF(AND(F31&gt;G31,COUNT(H12:H30)=0),B31,"")</f>
         <v/>
       </c>
     </row>
@@ -1793,7 +1793,7 @@
         <v/>
       </c>
       <c r="H32" s="14">
-        <f>IF(AND(F32&gt;G32,F31&lt;=G32),B32,"")</f>
+        <f>IF(AND(F32&gt;G32,COUNT(H12:H31)=0),B32,"")</f>
         <v/>
       </c>
     </row>
@@ -1861,7 +1861,7 @@
         <v/>
       </c>
       <c r="H35" s="14">
-        <f>IF(AND(F35&gt;G35,F34&lt;=G35),B35,"")</f>
+        <f>IF(AND(F35&gt;G35,COUNT(H34:H34)=0),B35,"")</f>
         <v/>
       </c>
     </row>
@@ -1895,7 +1895,7 @@
         <v/>
       </c>
       <c r="H36" s="14">
-        <f>IF(AND(F36&gt;G36,F35&lt;=G36),B36,"")</f>
+        <f>IF(AND(F36&gt;G36,COUNT(H34:H35)=0),B36,"")</f>
         <v/>
       </c>
     </row>
@@ -1929,7 +1929,7 @@
         <v/>
       </c>
       <c r="H37" s="14">
-        <f>IF(AND(F37&gt;G37,F36&lt;=G37),B37,"")</f>
+        <f>IF(AND(F37&gt;G37,COUNT(H34:H36)=0),B37,"")</f>
         <v/>
       </c>
     </row>
@@ -1963,7 +1963,7 @@
         <v/>
       </c>
       <c r="H38" s="14">
-        <f>IF(AND(F38&gt;G38,F37&lt;=G38),B38,"")</f>
+        <f>IF(AND(F38&gt;G38,COUNT(H34:H37)=0),B38,"")</f>
         <v/>
       </c>
     </row>
@@ -1997,7 +1997,7 @@
         <v/>
       </c>
       <c r="H39" s="14">
-        <f>IF(AND(F39&gt;G39,F38&lt;=G39),B39,"")</f>
+        <f>IF(AND(F39&gt;G39,COUNT(H34:H38)=0),B39,"")</f>
         <v/>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
         <v/>
       </c>
       <c r="H40" s="14">
-        <f>IF(AND(F40&gt;G40,F39&lt;=G40),B40,"")</f>
+        <f>IF(AND(F40&gt;G40,COUNT(H34:H39)=0),B40,"")</f>
         <v/>
       </c>
     </row>
@@ -2065,7 +2065,7 @@
         <v/>
       </c>
       <c r="H41" s="14">
-        <f>IF(AND(F41&gt;G41,F40&lt;=G41),B41,"")</f>
+        <f>IF(AND(F41&gt;G41,COUNT(H34:H40)=0),B41,"")</f>
         <v/>
       </c>
     </row>
@@ -2099,7 +2099,7 @@
         <v/>
       </c>
       <c r="H42" s="14">
-        <f>IF(AND(F42&gt;G42,F41&lt;=G42),B42,"")</f>
+        <f>IF(AND(F42&gt;G42,COUNT(H34:H41)=0),B42,"")</f>
         <v/>
       </c>
     </row>
@@ -2133,7 +2133,7 @@
         <v/>
       </c>
       <c r="H43" s="14">
-        <f>IF(AND(F43&gt;G43,F42&lt;=G43),B43,"")</f>
+        <f>IF(AND(F43&gt;G43,COUNT(H34:H42)=0),B43,"")</f>
         <v/>
       </c>
     </row>
@@ -2167,7 +2167,7 @@
         <v/>
       </c>
       <c r="H44" s="14">
-        <f>IF(AND(F44&gt;G44,F43&lt;=G44),B44,"")</f>
+        <f>IF(AND(F44&gt;G44,COUNT(H34:H43)=0),B44,"")</f>
         <v/>
       </c>
     </row>
@@ -2201,7 +2201,7 @@
         <v/>
       </c>
       <c r="H45" s="14">
-        <f>IF(AND(F45&gt;G45,F44&lt;=G45),B45,"")</f>
+        <f>IF(AND(F45&gt;G45,COUNT(H34:H44)=0),B45,"")</f>
         <v/>
       </c>
     </row>
@@ -2235,7 +2235,7 @@
         <v/>
       </c>
       <c r="H46" s="14">
-        <f>IF(AND(F46&gt;G46,F45&lt;=G46),B46,"")</f>
+        <f>IF(AND(F46&gt;G46,COUNT(H34:H45)=0),B46,"")</f>
         <v/>
       </c>
     </row>
@@ -2269,7 +2269,7 @@
         <v/>
       </c>
       <c r="H47" s="14">
-        <f>IF(AND(F47&gt;G47,F46&lt;=G47),B47,"")</f>
+        <f>IF(AND(F47&gt;G47,COUNT(H34:H46)=0),B47,"")</f>
         <v/>
       </c>
     </row>
@@ -2303,7 +2303,7 @@
         <v/>
       </c>
       <c r="H48" s="14">
-        <f>IF(AND(F48&gt;G48,F47&lt;=G48),B48,"")</f>
+        <f>IF(AND(F48&gt;G48,COUNT(H34:H47)=0),B48,"")</f>
         <v/>
       </c>
     </row>
@@ -2337,7 +2337,7 @@
         <v/>
       </c>
       <c r="H49" s="14">
-        <f>IF(AND(F49&gt;G49,F48&lt;=G49),B49,"")</f>
+        <f>IF(AND(F49&gt;G49,COUNT(H34:H48)=0),B49,"")</f>
         <v/>
       </c>
     </row>
@@ -2371,7 +2371,7 @@
         <v/>
       </c>
       <c r="H50" s="14">
-        <f>IF(AND(F50&gt;G50,F49&lt;=G50),B50,"")</f>
+        <f>IF(AND(F50&gt;G50,COUNT(H34:H49)=0),B50,"")</f>
         <v/>
       </c>
     </row>
@@ -2405,7 +2405,7 @@
         <v/>
       </c>
       <c r="H51" s="14">
-        <f>IF(AND(F51&gt;G51,F50&lt;=G51),B51,"")</f>
+        <f>IF(AND(F51&gt;G51,COUNT(H34:H50)=0),B51,"")</f>
         <v/>
       </c>
     </row>
@@ -2439,7 +2439,7 @@
         <v/>
       </c>
       <c r="H52" s="14">
-        <f>IF(AND(F52&gt;G52,F51&lt;=G52),B52,"")</f>
+        <f>IF(AND(F52&gt;G52,COUNT(H34:H51)=0),B52,"")</f>
         <v/>
       </c>
     </row>
@@ -2473,7 +2473,7 @@
         <v/>
       </c>
       <c r="H53" s="14">
-        <f>IF(AND(F53&gt;G53,F52&lt;=G53),B53,"")</f>
+        <f>IF(AND(F53&gt;G53,COUNT(H34:H52)=0),B53,"")</f>
         <v/>
       </c>
     </row>
@@ -2507,7 +2507,7 @@
         <v/>
       </c>
       <c r="H54" s="14">
-        <f>IF(AND(F54&gt;G54,F53&lt;=G54),B54,"")</f>
+        <f>IF(AND(F54&gt;G54,COUNT(H34:H53)=0),B54,"")</f>
         <v/>
       </c>
     </row>
@@ -2541,7 +2541,7 @@
         <v/>
       </c>
       <c r="H55" s="14">
-        <f>IF(AND(F55&gt;G55,F54&lt;=G55),B55,"")</f>
+        <f>IF(AND(F55&gt;G55,COUNT(H34:H54)=0),B55,"")</f>
         <v/>
       </c>
     </row>
@@ -2575,7 +2575,7 @@
         <v/>
       </c>
       <c r="H56" s="14">
-        <f>IF(AND(F56&gt;G56,F55&lt;=G56),B56,"")</f>
+        <f>IF(AND(F56&gt;G56,COUNT(H34:H55)=0),B56,"")</f>
         <v/>
       </c>
     </row>
@@ -2609,7 +2609,7 @@
         <v/>
       </c>
       <c r="H57" s="14">
-        <f>IF(AND(F57&gt;G57,F56&lt;=G57),B57,"")</f>
+        <f>IF(AND(F57&gt;G57,COUNT(H34:H56)=0),B57,"")</f>
         <v/>
       </c>
     </row>
@@ -2643,7 +2643,7 @@
         <v/>
       </c>
       <c r="H58" s="14">
-        <f>IF(AND(F58&gt;G58,F57&lt;=G58),B58,"")</f>
+        <f>IF(AND(F58&gt;G58,COUNT(H34:H57)=0),B58,"")</f>
         <v/>
       </c>
     </row>
@@ -2677,7 +2677,7 @@
         <v/>
       </c>
       <c r="H59" s="14">
-        <f>IF(AND(F59&gt;G59,F58&lt;=G59),B59,"")</f>
+        <f>IF(AND(F59&gt;G59,COUNT(H34:H58)=0),B59,"")</f>
         <v/>
       </c>
     </row>
@@ -2711,7 +2711,7 @@
         <v/>
       </c>
       <c r="H60" s="14">
-        <f>IF(AND(F60&gt;G60,F59&lt;=G60),B60,"")</f>
+        <f>IF(AND(F60&gt;G60,COUNT(H34:H59)=0),B60,"")</f>
         <v/>
       </c>
     </row>
@@ -2745,7 +2745,7 @@
         <v/>
       </c>
       <c r="H61" s="14">
-        <f>IF(AND(F61&gt;G61,F60&lt;=G61),B61,"")</f>
+        <f>IF(AND(F61&gt;G61,COUNT(H34:H60)=0),B61,"")</f>
         <v/>
       </c>
     </row>
@@ -2779,7 +2779,7 @@
         <v/>
       </c>
       <c r="H62" s="14">
-        <f>IF(AND(F62&gt;G62,F61&lt;=G62),B62,"")</f>
+        <f>IF(AND(F62&gt;G62,COUNT(H34:H61)=0),B62,"")</f>
         <v/>
       </c>
     </row>
@@ -2813,7 +2813,7 @@
         <v/>
       </c>
       <c r="H63" s="14">
-        <f>IF(AND(F63&gt;G63,F62&lt;=G63),B63,"")</f>
+        <f>IF(AND(F63&gt;G63,COUNT(H34:H62)=0),B63,"")</f>
         <v/>
       </c>
     </row>
@@ -2847,7 +2847,7 @@
         <v/>
       </c>
       <c r="H64" s="14">
-        <f>IF(AND(F64&gt;G64,F63&lt;=G64),B64,"")</f>
+        <f>IF(AND(F64&gt;G64,COUNT(H34:H63)=0),B64,"")</f>
         <v/>
       </c>
     </row>
@@ -2915,7 +2915,7 @@
         <v/>
       </c>
       <c r="H67" s="14">
-        <f>IF(AND(F67&gt;G67,F66&lt;=G67),B67,"")</f>
+        <f>IF(AND(F67&gt;G67,COUNT(H66:H66)=0),B67,"")</f>
         <v/>
       </c>
     </row>
@@ -2949,7 +2949,7 @@
         <v/>
       </c>
       <c r="H68" s="14">
-        <f>IF(AND(F68&gt;G68,F67&lt;=G68),B68,"")</f>
+        <f>IF(AND(F68&gt;G68,COUNT(H66:H67)=0),B68,"")</f>
         <v/>
       </c>
     </row>
@@ -2983,7 +2983,7 @@
         <v/>
       </c>
       <c r="H69" s="14">
-        <f>IF(AND(F69&gt;G69,F68&lt;=G69),B69,"")</f>
+        <f>IF(AND(F69&gt;G69,COUNT(H66:H68)=0),B69,"")</f>
         <v/>
       </c>
     </row>
@@ -3017,7 +3017,7 @@
         <v/>
       </c>
       <c r="H70" s="14">
-        <f>IF(AND(F70&gt;G70,F69&lt;=G70),B70,"")</f>
+        <f>IF(AND(F70&gt;G70,COUNT(H66:H69)=0),B70,"")</f>
         <v/>
       </c>
     </row>
@@ -3051,7 +3051,7 @@
         <v/>
       </c>
       <c r="H71" s="14">
-        <f>IF(AND(F71&gt;G71,F70&lt;=G71),B71,"")</f>
+        <f>IF(AND(F71&gt;G71,COUNT(H66:H70)=0),B71,"")</f>
         <v/>
       </c>
     </row>
@@ -3085,7 +3085,7 @@
         <v/>
       </c>
       <c r="H72" s="14">
-        <f>IF(AND(F72&gt;G72,F71&lt;=G72),B72,"")</f>
+        <f>IF(AND(F72&gt;G72,COUNT(H66:H71)=0),B72,"")</f>
         <v/>
       </c>
     </row>
@@ -3119,7 +3119,7 @@
         <v/>
       </c>
       <c r="H73" s="14">
-        <f>IF(AND(F73&gt;G73,F72&lt;=G73),B73,"")</f>
+        <f>IF(AND(F73&gt;G73,COUNT(H66:H72)=0),B73,"")</f>
         <v/>
       </c>
     </row>
@@ -3153,7 +3153,7 @@
         <v/>
       </c>
       <c r="H74" s="14">
-        <f>IF(AND(F74&gt;G74,F73&lt;=G74),B74,"")</f>
+        <f>IF(AND(F74&gt;G74,COUNT(H66:H73)=0),B74,"")</f>
         <v/>
       </c>
     </row>
@@ -3187,7 +3187,7 @@
         <v/>
       </c>
       <c r="H75" s="14">
-        <f>IF(AND(F75&gt;G75,F74&lt;=G75),B75,"")</f>
+        <f>IF(AND(F75&gt;G75,COUNT(H66:H74)=0),B75,"")</f>
         <v/>
       </c>
     </row>
@@ -3221,7 +3221,7 @@
         <v/>
       </c>
       <c r="H76" s="14">
-        <f>IF(AND(F76&gt;G76,F75&lt;=G76),B76,"")</f>
+        <f>IF(AND(F76&gt;G76,COUNT(H66:H75)=0),B76,"")</f>
         <v/>
       </c>
     </row>
@@ -3255,7 +3255,7 @@
         <v/>
       </c>
       <c r="H77" s="14">
-        <f>IF(AND(F77&gt;G77,F76&lt;=G77),B77,"")</f>
+        <f>IF(AND(F77&gt;G77,COUNT(H66:H76)=0),B77,"")</f>
         <v/>
       </c>
     </row>
@@ -3289,7 +3289,7 @@
         <v/>
       </c>
       <c r="H78" s="14">
-        <f>IF(AND(F78&gt;G78,F77&lt;=G78),B78,"")</f>
+        <f>IF(AND(F78&gt;G78,COUNT(H66:H77)=0),B78,"")</f>
         <v/>
       </c>
     </row>
@@ -3323,7 +3323,7 @@
         <v/>
       </c>
       <c r="H79" s="14">
-        <f>IF(AND(F79&gt;G79,F78&lt;=G79),B79,"")</f>
+        <f>IF(AND(F79&gt;G79,COUNT(H66:H78)=0),B79,"")</f>
         <v/>
       </c>
     </row>
@@ -3357,7 +3357,7 @@
         <v/>
       </c>
       <c r="H80" s="14">
-        <f>IF(AND(F80&gt;G80,F79&lt;=G80),B80,"")</f>
+        <f>IF(AND(F80&gt;G80,COUNT(H66:H79)=0),B80,"")</f>
         <v/>
       </c>
     </row>
@@ -3391,7 +3391,7 @@
         <v/>
       </c>
       <c r="H81" s="14">
-        <f>IF(AND(F81&gt;G81,F80&lt;=G81),B81,"")</f>
+        <f>IF(AND(F81&gt;G81,COUNT(H66:H80)=0),B81,"")</f>
         <v/>
       </c>
     </row>
@@ -3425,7 +3425,7 @@
         <v/>
       </c>
       <c r="H82" s="14">
-        <f>IF(AND(F82&gt;G82,F81&lt;=G82),B82,"")</f>
+        <f>IF(AND(F82&gt;G82,COUNT(H66:H81)=0),B82,"")</f>
         <v/>
       </c>
     </row>
@@ -3459,7 +3459,7 @@
         <v/>
       </c>
       <c r="H83" s="14">
-        <f>IF(AND(F83&gt;G83,F82&lt;=G83),B83,"")</f>
+        <f>IF(AND(F83&gt;G83,COUNT(H66:H82)=0),B83,"")</f>
         <v/>
       </c>
     </row>
@@ -3493,7 +3493,7 @@
         <v/>
       </c>
       <c r="H84" s="14">
-        <f>IF(AND(F84&gt;G84,F83&lt;=G84),B84,"")</f>
+        <f>IF(AND(F84&gt;G84,COUNT(H66:H83)=0),B84,"")</f>
         <v/>
       </c>
     </row>
@@ -3527,7 +3527,7 @@
         <v/>
       </c>
       <c r="H85" s="14">
-        <f>IF(AND(F85&gt;G85,F84&lt;=G85),B85,"")</f>
+        <f>IF(AND(F85&gt;G85,COUNT(H66:H84)=0),B85,"")</f>
         <v/>
       </c>
     </row>
@@ -3561,7 +3561,7 @@
         <v/>
       </c>
       <c r="H86" s="14">
-        <f>IF(AND(F86&gt;G86,F85&lt;=G86),B86,"")</f>
+        <f>IF(AND(F86&gt;G86,COUNT(H66:H85)=0),B86,"")</f>
         <v/>
       </c>
     </row>
@@ -3598,7 +3598,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Decision variables are preloaded to the audited optimum and remain Solver-ready.</t>
+          <t>Decision variables are preloaded to the audited optimum; desktop Excel Solver inputs are listed below.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Strengthen workbook input and labor formulas
Co-authored-by: bvn2103 <318941354+bvn2103@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/capabilities/marginal-analysis/model.xlsx
+++ b/capabilities/marginal-analysis/model.xlsx
@@ -22,20 +22,20 @@
     <definedName name="Fixed_Cost">Inputs!$B$9</definedName>
     <definedName name="Total_Bed_Cap">Inputs!$B$10</definedName>
     <definedName name="Tomato_Base_Hours_Per_Week">Inputs!$B$13</definedName>
-    <definedName name="Tomato_Dim_Pct">Inputs!$C$13</definedName>
-    <definedName name="Tomato_Revenue_Per_Bed">Inputs!$D$13</definedName>
-    <definedName name="Tomato_Fertilizer_Per_Bed">Inputs!$E$13</definedName>
-    <definedName name="Tomato_Max_Beds">Inputs!$F$13</definedName>
+    <definedName name="Tomato_Dim_Pct">Inputs!$D$13</definedName>
+    <definedName name="Tomato_Revenue_Per_Bed">Inputs!$F$13</definedName>
+    <definedName name="Tomato_Fertilizer_Per_Bed">Inputs!$H$13</definedName>
+    <definedName name="Tomato_Max_Beds">Inputs!$J$13</definedName>
     <definedName name="Mesclun_Base_Hours_Per_Week">Inputs!$B$14</definedName>
-    <definedName name="Mesclun_Dim_Pct">Inputs!$C$14</definedName>
-    <definedName name="Mesclun_Revenue_Per_Bed">Inputs!$D$14</definedName>
-    <definedName name="Mesclun_Fertilizer_Per_Bed">Inputs!$E$14</definedName>
-    <definedName name="Mesclun_Max_Beds">Inputs!$F$14</definedName>
+    <definedName name="Mesclun_Dim_Pct">Inputs!$D$14</definedName>
+    <definedName name="Mesclun_Revenue_Per_Bed">Inputs!$F$14</definedName>
+    <definedName name="Mesclun_Fertilizer_Per_Bed">Inputs!$H$14</definedName>
+    <definedName name="Mesclun_Max_Beds">Inputs!$J$14</definedName>
     <definedName name="Carrot_Base_Hours_Per_Week">Inputs!$B$15</definedName>
-    <definedName name="Carrot_Dim_Pct">Inputs!$C$15</definedName>
-    <definedName name="Carrot_Revenue_Per_Bed">Inputs!$D$15</definedName>
-    <definedName name="Carrot_Fertilizer_Per_Bed">Inputs!$E$15</definedName>
-    <definedName name="Carrot_Max_Beds">Inputs!$F$15</definedName>
+    <definedName name="Carrot_Dim_Pct">Inputs!$D$15</definedName>
+    <definedName name="Carrot_Revenue_Per_Bed">Inputs!$F$15</definedName>
+    <definedName name="Carrot_Fertilizer_Per_Bed">Inputs!$H$15</definedName>
+    <definedName name="Carrot_Max_Beds">Inputs!$J$15</definedName>
     <definedName name="Schedule_Crop">'Labor &amp; Cost'!$A$12:$A$86</definedName>
     <definedName name="Schedule_Q">'Labor &amp; Cost'!$B$12:$B$86</definedName>
     <definedName name="Schedule_Total_Labor">'Labor &amp; Cost'!$C$12:$C$86</definedName>
@@ -584,18 +584,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:O15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -633,7 +638,7 @@
           <t>Source / notes</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>Published reference checks</t>
         </is>
@@ -658,12 +663,12 @@
           <t>Case scenario</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="N4" s="5" t="inlineStr">
         <is>
           <t>Optimal mix</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="O4" s="3" t="inlineStr">
         <is>
           <t>Tomatoes 10, Mesclun 30, Carrots 20</t>
         </is>
@@ -688,12 +693,12 @@
           <t>Case scenario; consumed before temporary labor</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="N5" s="5" t="inlineStr">
         <is>
           <t>Published season profit</t>
         </is>
       </c>
-      <c r="J5" s="6" t="n">
+      <c r="O5" s="6" t="n">
         <v>42762</v>
       </c>
     </row>
@@ -716,12 +721,12 @@
           <t>Opportunity cost from case scenario</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="N6" s="5" t="inlineStr">
         <is>
           <t>Exact script profit</t>
         </is>
       </c>
-      <c r="J6" s="6" t="n">
+      <c r="O6" s="6" t="n">
         <v>42768.32825620536</v>
       </c>
     </row>
@@ -813,30 +818,55 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Base hrs/week/bed</t>
+          <t>Base value</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
+          <t>Base unit</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
           <t>DIM_PCT</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Revenue/bed</t>
-        </is>
-      </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Fertilizer/bed</t>
+          <t>DIM unit</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
+          <t>Revenue value</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Revenue unit</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Fertilizer value</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Fertilizer unit</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
           <t>Max beds</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Max unit</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>Source / notes</t>
         </is>
@@ -851,19 +881,44 @@
       <c r="B13" s="7" t="n">
         <v>2.5</v>
       </c>
-      <c r="C13" s="8" t="n">
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>hours/week/bed</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="n">
         <v>0.1</v>
       </c>
-      <c r="D13" s="6" t="n">
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="n">
         <v>8800</v>
       </c>
-      <c r="E13" s="6" t="n">
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>$/bed</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="n">
         <v>880</v>
       </c>
-      <c r="F13" s="9" t="n">
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>$/bed</t>
+        </is>
+      </c>
+      <c r="J13" s="9" t="n">
         <v>20</v>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>beds</t>
+        </is>
+      </c>
+      <c r="L13" s="3" t="inlineStr">
         <is>
           <t>2.50 hours/week/bed</t>
         </is>
@@ -878,19 +933,44 @@
       <c r="B14" s="7" t="n">
         <v>1.25</v>
       </c>
-      <c r="C14" s="8" t="n">
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>hours/week/bed</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="n">
         <v>0.0125</v>
       </c>
-      <c r="D14" s="6" t="n">
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="n">
         <v>2700</v>
       </c>
-      <c r="E14" s="6" t="n">
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>$/bed</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="n">
         <v>880</v>
       </c>
-      <c r="F14" s="9" t="n">
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>$/bed</t>
+        </is>
+      </c>
+      <c r="J14" s="9" t="n">
         <v>30</v>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>beds</t>
+        </is>
+      </c>
+      <c r="L14" s="3" t="inlineStr">
         <is>
           <t>1.25 hours/week/bed</t>
         </is>
@@ -906,19 +986,44 @@
         <f>5/6</f>
         <v/>
       </c>
-      <c r="C15" s="8" t="n">
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>hours/week/bed</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="n">
         <v>0.025</v>
       </c>
-      <c r="D15" s="6" t="n">
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="n">
         <v>2094</v>
       </c>
-      <c r="E15" s="6" t="n">
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>$/bed</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="n">
         <v>440</v>
       </c>
-      <c r="F15" s="9" t="n">
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>$/bed</t>
+        </is>
+      </c>
+      <c r="J15" s="9" t="n">
         <v>20</v>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>beds</t>
+        </is>
+      </c>
+      <c r="L15" s="3" t="inlineStr">
         <is>
           <t>Exact case value 2.5/3 hours/week/bed</t>
         </is>
@@ -3649,7 +3754,7 @@
         <v>10</v>
       </c>
       <c r="C4" s="13">
-        <f>SUMIFS(Schedule_Total_Labor,Schedule_Crop,A4,Schedule_Q,B4)</f>
+        <f>IF(B4=0,0,Tomato_Base_Hours_Per_Week*Season_Weeks*B4*(1+Tomato_Dim_Pct)^B4)</f>
         <v/>
       </c>
       <c r="D4" s="10">
@@ -3679,7 +3784,7 @@
         <v>30</v>
       </c>
       <c r="C5" s="13">
-        <f>SUMIFS(Schedule_Total_Labor,Schedule_Crop,A5,Schedule_Q,B5)</f>
+        <f>IF(B5=0,0,Mesclun_Base_Hours_Per_Week*Season_Weeks*B5*(1+Mesclun_Dim_Pct)^B5)</f>
         <v/>
       </c>
       <c r="D5" s="10">
@@ -3709,7 +3814,7 @@
         <v>20</v>
       </c>
       <c r="C6" s="13">
-        <f>SUMIFS(Schedule_Total_Labor,Schedule_Crop,A6,Schedule_Q,B6)</f>
+        <f>IF(B6=0,0,Carrot_Base_Hours_Per_Week*Season_Weeks*B6*(1+Carrot_Dim_Pct)^B6)</f>
         <v/>
       </c>
       <c r="D6" s="10">

</xml_diff>